<commit_message>
Rename workflow and update container settings fd9382e68d875c844d462c13cbb858a2f875470b
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-core-appointment.xlsx
+++ b/main/ig/StructureDefinition-fr-core-appointment.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-12T14:35:23+00:00</t>
+    <t>2026-06-26T12:32:04+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -815,7 +815,7 @@
     <t>The style of appointment or patient that has been booked in the slot (not service type).</t>
   </si>
   <si>
-    <t>http://terminology.hl7.org/ValueSet/v2-0276|2.9</t>
+    <t>http://terminology.hl7.org/ValueSet/v2-0276|3.0.0</t>
   </si>
   <si>
     <t>.code</t>

</xml_diff>